<commit_message>
Añadir actividad: Entrega de Certificados Diplomatura Programación
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q27"/>
+  <dimension ref="A1:Q28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2036,7 +2036,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t>ALTA</t>
@@ -2091,7 +2095,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t>ALTA</t>
@@ -2135,14 +2143,22 @@
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>ALTA</t>
@@ -2161,7 +2177,11 @@
           <t>Cipolletti</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr"/>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Sin especificar</t>
+        </is>
+      </c>
       <c r="P26" t="inlineStr">
         <is>
           <t>Capacitación para el armado y el uso de las Maquetas V4LE.</t>
@@ -2186,14 +2206,22 @@
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
           <t>ALTA</t>
@@ -2212,7 +2240,11 @@
           <t>General Roca</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr"/>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Sin especificar</t>
+        </is>
+      </c>
       <c r="P27" t="inlineStr">
         <is>
           <t>Capacitación para docentes para el armado y uso de las Maquetas V4LE.</t>
@@ -2220,6 +2252,65 @@
       </c>
       <c r="Q27" t="n">
         <v>50</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>36</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entrega de Certificados Diplomatura Programación </t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Estudiantes Programación Roca y familias</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Gral. Roca</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>CET 33- Auditorio</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Entrega de los 12 certificados de los estudiantes de Roca que no acudieron a la Jornada.</t>
+        </is>
+      </c>
+      <c r="Q28" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Añadir actividad: Entrega de maqueta ESRN 151 de Roca
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q28"/>
+  <dimension ref="A1:Q29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2269,7 +2269,11 @@
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
@@ -2313,6 +2317,61 @@
         <v>20</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>42</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Entrega de maqueta ESRN 151 de Roca</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Gral. Roca</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>ESRN 151</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entrega de maqueta y actividad con los profes </t>
+        </is>
+      </c>
+      <c r="Q29" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Añadir actividad: Soy Río Negro y RíoBot 2.0
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q29"/>
+  <dimension ref="A1:Q30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2332,14 +2332,22 @@
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr">
         <is>
           <t>ALTA</t>
@@ -2372,6 +2380,57 @@
         <v>50</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>42</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Soy Río Negro y RíoBot 2.0</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>General Roca</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Asociación Española - España 1371</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="n">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Añadir actividad: Aula Hidroponica
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q30"/>
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2431,6 +2431,65 @@
         <v>100</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>42</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Aula Hidroponica</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>UNCo</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Cinco Saltos</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Facultad de Ciencias Agrarias</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Inauguración del AULA HIDROPONICA</t>
+        </is>
+      </c>
+      <c r="Q31" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Añadir actividad: JOVEN FEST RN
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q31"/>
+  <dimension ref="A1:Q32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2490,6 +2490,65 @@
         <v>50</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>42</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>JOVEN FEST RN</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Secretaría de Juventud</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>General Roca</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>ESRN 9</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Participación del evento con la charla "Vocaciones en el Río Negro que se viene", Maquetas V4LE y portal Tu Vocación.</t>
+        </is>
+      </c>
+      <c r="Q32" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Modificar actividad: Soy Río Negro y RíoBot 2.0
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -2395,7 +2395,11 @@
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Modernización | Gobierno de Río Negro</t>
+        </is>
+      </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Añadir actividad: “Microbrew.AR: IA aplicada a la tecnología cervecera”
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q32"/>
+  <dimension ref="A1:Q33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2406,7 +2406,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
           <t>ALTA</t>
@@ -2461,7 +2465,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>ALTA</t>
@@ -2520,7 +2528,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr">
         <is>
           <t>ALTA</t>
@@ -2553,6 +2565,69 @@
         <v>50</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>45</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>“Microbrew.AR: IA aplicada a la tecnología cervecera”</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IPATEC </t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Cerveceros</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Viedma</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>CURZAS</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>En el marco del proyecto de extensión universitaria “Microbrew.AR: IA aplicada a la tecnología cervecera”, desarrollado por el IPATEC (CONICET–Universidad Nacional del Comahue), se realizarán jornadas de capacitación destinadas a productores cerveceros de distintas regiones de Río Negro.</t>
+        </is>
+      </c>
+      <c r="Q33" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Añadir actividad: UNRN gestando cambios en la esquila
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q34"/>
+  <dimension ref="A1:Q35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2691,6 +2691,61 @@
         <v>50</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-11-12</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>46</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>UNRN gestando cambios en la esquila</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UNRN </t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Sin especificar</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Maquinchao</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Proyecto de extensión propone implementar un programa integral de capacitación y microacreditación participativa en esquila y acondicionamiento ovino sustentable, con eje en la prevención de lesiones (kinefilaxia), el bienestar animal, la sustentabilidad ambiental y la valorización de la lana. Se articula con PROLANA Río Negro, el Ministerio de Producción y Agroindustria, SENASA, INTA, el Ente Región Sur, cooperativas ovinas y la Lavadora de Lana de Ñorquinco.</t>
+        </is>
+      </c>
+      <c r="Q35" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Eliminar actividad fila 33
</commit_message>
<xml_diff>
--- a/agenda_territorial_consolidada.xlsx
+++ b/agenda_territorial_consolidada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q39"/>
+  <dimension ref="A1:Q38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2694,7 +2694,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-11-12</t>
+          <t>2026-11-13</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2708,7 +2708,7 @@
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">UNRN </t>
+          <t>UNRN</t>
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
@@ -2717,7 +2717,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr">
         <is>
           <t>ALTA</t>
@@ -2736,10 +2740,14 @@
           <t>Maquinchao</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr"/>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Sin especificar</t>
+        </is>
+      </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>Proyecto de extensión propone implementar un programa integral de capacitación y microacreditación participativa en esquila y acondicionamiento ovino sustentable, con eje en la prevención de lesiones (kinefilaxia), el bienestar animal, la sustentabilidad ambiental y la valorización de la lana. Se articula con PROLANA Río Negro, el Ministerio de Producción y Agroindustria, SENASA, INTA, el Ente Región Sur, cooperativas ovinas y la Lavadora de Lana de Ñorquinco.</t>
+          <t>Proyecto de extensión que propone implementar un programa integral de capacitación y microacreditación participativa en esquila y acondicionamiento ovino sustentable, con eje en la prevención de lesiones (kinefilaxia), el bienestar animal, la sustentabilidad ambiental y la valorización de la lana. Se articula con PROLANA Río Negro, el Ministerio de Producción y Agroindustria, SENASA, INTA, el Ente Región Sur, cooperativas ovinas y la Lavadora de Lana de Ñorquinco.</t>
         </is>
       </c>
       <c r="Q35" t="n">
@@ -2749,11 +2757,11 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-11-13</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -2772,7 +2780,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr">
         <is>
           <t>ALTA</t>
@@ -2783,18 +2795,22 @@
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr">
         <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Maquinchao</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
           <t>Sin especificar</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>Maquinchao</t>
-        </is>
-      </c>
-      <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
         <is>
-          <t>Proyecto de extensión que propone implementar un programa integral de capacitación y microacreditación participativa en esquila y acondicionamiento ovino sustentable, con eje en la prevención de lesiones (kinefilaxia), el bienestar animal, la sustentabilidad ambiental y la valorización de la lana. Se articula con PROLANA Río Negro, el Ministerio de Producción y Agroindustria, SENASA, INTA, el Ente Región Sur, cooperativas ovinas y la Lavadora de Lana de Ñorquinco.</t>
+          <t>Proyecto de extensión propone implementar un programa integral de capacitación y microacreditación participativa en esquila y acondicionamiento ovino sustentable, con eje en la prevención de lesiones (kinefilaxia), el bienestar animal, la sustentabilidad ambiental y la valorización de la lana. Se articula con PROLANA Río Negro, el Ministerio de Producción y Agroindustria, SENASA, INTA, el Ente Región Sur, cooperativas ovinas y la Lavadora de Lana de Ñorquinco.</t>
         </is>
       </c>
       <c r="Q36" t="n">
@@ -2804,7 +2820,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-11-20</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2827,7 +2843,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr">
         <is>
           <t>ALTA</t>
@@ -2838,7 +2858,7 @@
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2846,7 +2866,11 @@
           <t>Maquinchao</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr"/>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Sin especificar</t>
+        </is>
+      </c>
       <c r="P37" t="inlineStr">
         <is>
           <t>Proyecto de extensión propone implementar un programa integral de capacitación y microacreditación participativa en esquila y acondicionamiento ovino sustentable, con eje en la prevención de lesiones (kinefilaxia), el bienestar animal, la sustentabilidad ambiental y la valorización de la lana. Se articula con PROLANA Río Negro, el Ministerio de Producción y Agroindustria, SENASA, INTA, el Ente Región Sur, cooperativas ovinas y la Lavadora de Lana de Ñorquinco.</t>
@@ -2859,7 +2883,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-11-20</t>
+          <t>2026-11-21</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -2882,7 +2906,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr">
         <is>
           <t>ALTA</t>
@@ -2901,68 +2929,17 @@
           <t>Maquinchao</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr"/>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Sin especificar</t>
+        </is>
+      </c>
       <c r="P38" t="inlineStr">
         <is>
           <t>Proyecto de extensión propone implementar un programa integral de capacitación y microacreditación participativa en esquila y acondicionamiento ovino sustentable, con eje en la prevención de lesiones (kinefilaxia), el bienestar animal, la sustentabilidad ambiental y la valorización de la lana. Se articula con PROLANA Río Negro, el Ministerio de Producción y Agroindustria, SENASA, INTA, el Ente Región Sur, cooperativas ovinas y la Lavadora de Lana de Ñorquinco.</t>
         </is>
       </c>
       <c r="Q38" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>2026-11-21</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>47</v>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>UNRN gestando cambios en la esquila</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>UNRN</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>Sin especificar</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>Maquinchao</t>
-        </is>
-      </c>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr">
-        <is>
-          <t>Proyecto de extensión propone implementar un programa integral de capacitación y microacreditación participativa en esquila y acondicionamiento ovino sustentable, con eje en la prevención de lesiones (kinefilaxia), el bienestar animal, la sustentabilidad ambiental y la valorización de la lana. Se articula con PROLANA Río Negro, el Ministerio de Producción y Agroindustria, SENASA, INTA, el Ente Región Sur, cooperativas ovinas y la Lavadora de Lana de Ñorquinco.</t>
-        </is>
-      </c>
-      <c r="Q39" t="n">
         <v>50</v>
       </c>
     </row>

</xml_diff>